<commit_message>
Add recommendations visuals and validation
</commit_message>
<xml_diff>
--- a/outputs/trader_sentiment_analysis/trader_sentiment_analysis.xlsx
+++ b/outputs/trader_sentiment_analysis/trader_sentiment_analysis.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="R222c121cdb0549ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sentiment Summary" sheetId="2" r:id="R8a5dd1b5da594990"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Direction Plays" sheetId="3" r:id="Re41a4e8359104f68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Trend" sheetId="4" r:id="R8379b9bc54e34752"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top Coins" sheetId="5" r:id="Rc044136a00074412"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account Edges" sheetId="6" r:id="R78f651a296244552"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="7" r:id="Re942b1f9d0b946aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="Reff845f513e44f01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sentiment Summary" sheetId="2" r:id="R93945c5cc7c44585"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Direction Plays" sheetId="3" r:id="Reb2a5b6804754406"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Trend" sheetId="4" r:id="Re287394f50044e17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top Coins" sheetId="5" r:id="R0bf982465c12477d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account Edges" sheetId="6" r:id="R8df530f1144642ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="7" r:id="R15085bc6f8cc4257"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stat Validation" sheetId="8" r:id="Rf0f321645d18478a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +27,7 @@
     <x:numFmt numFmtId="203" formatCode="$#,##0.00"/>
     <x:numFmt numFmtId="204" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -76,8 +77,14 @@
       <x:color rgb="FF0B1320"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="20"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="14">
+  <x:fills count="22">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -144,51 +151,76 @@
         <x:fgColor rgb="FFF7F9FC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1320"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B2A41"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF19324A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1320"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B2A41"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF19324A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="19">
+  <x:borders count="37">
     <x:border/>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
     <x:border>
       <x:right/>
       <x:bottom/>
@@ -235,7 +267,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="89">
+  <x:cellXfs count="161">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -381,6 +413,158 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="17" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="17" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="17" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="17" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="17" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="17" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="21" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="21" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="21" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="21" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="21" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="21" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -670,7 +854,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra87702b8a7d64d7a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4b09ab3413524ff2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -700,7 +884,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R675fb3c6463c4b06"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R46e8ae6ca9b04297"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -833,6 +1017,24 @@
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Detail"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="StatisticalValidation" displayName="StatisticalValidation" ref="A5:J10" headerRowCount="1">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="sentiment"/>
+    <x:tableColumn id="2" name="days_observed"/>
+    <x:tableColumn id="3" name="mean_daily_net_pnl"/>
+    <x:tableColumn id="4" name="mean_daily_net_pnl_ci_low"/>
+    <x:tableColumn id="5" name="mean_daily_net_pnl_ci_high"/>
+    <x:tableColumn id="6" name="mean_daily_pnl_per_1k_volume"/>
+    <x:tableColumn id="7" name="mean_daily_pnl_per_1k_ci_low"/>
+    <x:tableColumn id="8" name="mean_daily_pnl_per_1k_ci_high"/>
+    <x:tableColumn id="9" name="mean_daily_win_rate"/>
+    <x:tableColumn id="10" name="interpretation"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -1493,9 +1695,9 @@
     <x:mergeCell ref="A30:F32"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe09b23c3e4647bb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd75cab3615444cbf"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9934b17e0cfc4c09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c9500e7586b46a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1858,7 +2060,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re85ef73f59eb4886"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73a458cbedb446c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5047,7 +5249,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcffe44f71cc3448c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc65a2bd54c1a4f2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31732,7 +31934,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra95ca138e83042b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e48643bd1a74e58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33482,7 +33684,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0f8d7b9f5aa4727"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ea329e0b2a1439f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34266,7 +34468,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bb0d1804b4c45cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc148e549f3ac4bf6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34376,7 +34578,237 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R778354f6b6a04895"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc425bb277a6466c"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="45" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="25.5" customHeight="1">
+      <x:c r="A1" s="127" t="str">
+        <x:v>Statistical Validation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="21" customHeight="1">
+      <x:c r="A2" s="131" t="str">
+        <x:v>Bootstrap confidence intervals for daily regime efficiency. These checks support regime filtering, but do not prove causality.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="31.5" customHeight="1">
+      <x:c r="A5" s="135" t="str">
+        <x:v>Sentiment</x:v>
+      </x:c>
+      <x:c r="B5" s="135" t="str">
+        <x:v>Days</x:v>
+      </x:c>
+      <x:c r="C5" s="135" t="str">
+        <x:v>Mean Daily Net PnL</x:v>
+      </x:c>
+      <x:c r="D5" s="135" t="str">
+        <x:v>Net PnL CI Low</x:v>
+      </x:c>
+      <x:c r="E5" s="135" t="str">
+        <x:v>Net PnL CI High</x:v>
+      </x:c>
+      <x:c r="F5" s="135" t="str">
+        <x:v>Mean Daily PnL / $1k</x:v>
+      </x:c>
+      <x:c r="G5" s="135" t="str">
+        <x:v>PnL / $1k CI Low</x:v>
+      </x:c>
+      <x:c r="H5" s="135" t="str">
+        <x:v>PnL / $1k CI High</x:v>
+      </x:c>
+      <x:c r="I5" s="135" t="str">
+        <x:v>Mean Daily Win Rate</x:v>
+      </x:c>
+      <x:c r="J5" s="135" t="str">
+        <x:v>Validation Takeaway</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="25.5" customHeight="1">
+      <x:c r="A6" s="146" t="str">
+        <x:v>Extreme Fear</x:v>
+      </x:c>
+      <x:c r="B6" s="147" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C6" s="155" t="n">
+        <x:v>51087.25818218665</x:v>
+      </x:c>
+      <x:c r="D6" s="155" t="n">
+        <x:v>6034.294345995668</x:v>
+      </x:c>
+      <x:c r="E6" s="155" t="n">
+        <x:v>106078.05726834146</x:v>
+      </x:c>
+      <x:c r="F6" s="155" t="n">
+        <x:v>7.595179907057886</x:v>
+      </x:c>
+      <x:c r="G6" s="155" t="n">
+        <x:v>-3.128833588565914</x:v>
+      </x:c>
+      <x:c r="H6" s="155" t="n">
+        <x:v>19.64494595594519</x:v>
+      </x:c>
+      <x:c r="I6" s="158" t="n">
+        <x:v>0.6544334990141908</x:v>
+      </x:c>
+      <x:c r="J6" s="148" t="str">
+        <x:v>bootstrap interval crossed zero; treat edge as less stable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="25.5" customHeight="1">
+      <x:c r="A7" s="149" t="str">
+        <x:v>Fear</x:v>
+      </x:c>
+      <x:c r="B7" s="150" t="n">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C7" s="156" t="n">
+        <x:v>35875.80761503126</x:v>
+      </x:c>
+      <x:c r="D7" s="156" t="n">
+        <x:v>19202.466447999293</x:v>
+      </x:c>
+      <x:c r="E7" s="156" t="n">
+        <x:v>56180.885293136336</x:v>
+      </x:c>
+      <x:c r="F7" s="156" t="n">
+        <x:v>8.801228558548559</x:v>
+      </x:c>
+      <x:c r="G7" s="156" t="n">
+        <x:v>1.6433010860241448</x:v>
+      </x:c>
+      <x:c r="H7" s="156" t="n">
+        <x:v>16.42664022058799</x:v>
+      </x:c>
+      <x:c r="I7" s="159" t="n">
+        <x:v>0.8807139342598307</x:v>
+      </x:c>
+      <x:c r="J7" s="151" t="str">
+        <x:v>daily efficiency stayed positive in bootstrap interval</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="25.5" customHeight="1">
+      <x:c r="A8" s="149" t="str">
+        <x:v>Neutral</x:v>
+      </x:c>
+      <x:c r="B8" s="150" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="C8" s="156" t="n">
+        <x:v>18709.64786934521</x:v>
+      </x:c>
+      <x:c r="D8" s="156" t="n">
+        <x:v>10499.311597402977</x:v>
+      </x:c>
+      <x:c r="E8" s="156" t="n">
+        <x:v>28545.05459893593</x:v>
+      </x:c>
+      <x:c r="F8" s="156" t="n">
+        <x:v>7.3455691192757255</x:v>
+      </x:c>
+      <x:c r="G8" s="156" t="n">
+        <x:v>-1.2711363557522666</x:v>
+      </x:c>
+      <x:c r="H8" s="156" t="n">
+        <x:v>16.71550629950772</x:v>
+      </x:c>
+      <x:c r="I8" s="159" t="n">
+        <x:v>0.7937897168589675</x:v>
+      </x:c>
+      <x:c r="J8" s="151" t="str">
+        <x:v>bootstrap interval crossed zero; treat edge as less stable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="25.5" customHeight="1">
+      <x:c r="A9" s="149" t="str">
+        <x:v>Greed</x:v>
+      </x:c>
+      <x:c r="B9" s="150" t="n">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="C9" s="156" t="n">
+        <x:v>10813.629953221925</x:v>
+      </x:c>
+      <x:c r="D9" s="156" t="n">
+        <x:v>2428.1435908965686</x:v>
+      </x:c>
+      <x:c r="E9" s="156" t="n">
+        <x:v>20112.907327396697</x:v>
+      </x:c>
+      <x:c r="F9" s="156" t="n">
+        <x:v>9.533095187934107</x:v>
+      </x:c>
+      <x:c r="G9" s="156" t="n">
+        <x:v>5.3766355705449635</x:v>
+      </x:c>
+      <x:c r="H9" s="156" t="n">
+        <x:v>14.53266531505959</x:v>
+      </x:c>
+      <x:c r="I9" s="159" t="n">
+        <x:v>0.8130205397780562</x:v>
+      </x:c>
+      <x:c r="J9" s="151" t="str">
+        <x:v>daily efficiency stayed positive in bootstrap interval</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="25.5" customHeight="1">
+      <x:c r="A10" s="152" t="str">
+        <x:v>Extreme Greed</x:v>
+      </x:c>
+      <x:c r="B10" s="153" t="n">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="C10" s="157" t="n">
+        <x:v>23580.181098314475</x:v>
+      </x:c>
+      <x:c r="D10" s="157" t="n">
+        <x:v>12095.25098283465</x:v>
+      </x:c>
+      <x:c r="E10" s="157" t="n">
+        <x:v>37819.16804812924</x:v>
+      </x:c>
+      <x:c r="F10" s="157" t="n">
+        <x:v>20.812368687511125</x:v>
+      </x:c>
+      <x:c r="G10" s="157" t="n">
+        <x:v>12.297859390458841</x:v>
+      </x:c>
+      <x:c r="H10" s="157" t="n">
+        <x:v>32.03014532785603</x:v>
+      </x:c>
+      <x:c r="I10" s="160" t="n">
+        <x:v>0.8865331257591066</x:v>
+      </x:c>
+      <x:c r="J10" s="154" t="str">
+        <x:v>daily efficiency stayed positive in bootstrap interval</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd95718236fb54d3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>